<commit_message>
data: refresh from Google Sheet
</commit_message>
<xml_diff>
--- a/data/hep-tracking.xlsx
+++ b/data/hep-tracking.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Organization</t>
   </si>
@@ -91,6 +91,28 @@
   </si>
   <si>
     <t>Lorem ipsum dolor sit amet consectetur adipiscing elit. Quisque faucibus ex sapien vitae pellentesque sem placerat. In id cursus mi pretium tellus duis convallis. Tempus leo eu aenean sed diam urna tempor. Pulvinar vivamus fringilla lacus nec metus bibendum egestas. Iaculis massa nisl malesuada lacinia integer nunc posuere. Ut hendrerit semper vel class aptent taciti sociosqu. Ad litora torquent per conubia nostra inceptos himenaeos.</t>
+  </si>
+  <si>
+    <t>Momo</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF76A5AF"/>
+      </rPr>
+      <t>Lorem ipsum dolor sit amet consectetur a</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t>dipiscing elit. Quisque faucibus ex sapien vitae pellentesque sem placerat. In id cursus mi pretium tellus duis convallis. Tempus leo eu aenean sed diam urna tempor. Pulvinar vivamus fringilla lacus nec metus bibendum egestas. Iaculis massa nisl malesuada lacinia integer nunc posuere. Ut hendrerit semper vel class aptent taciti sociosqu. Ad litora torquent per conubia nostra inceptos himenaeos.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -407,6 +429,20 @@
         <v>12</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2030.0</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>